<commit_message>
refined the code for the stats groups and started working on the table
</commit_message>
<xml_diff>
--- a/excel files/ISWE_Best_practices-parallelism_merged (1).xlsx
+++ b/excel files/ISWE_Best_practices-parallelism_merged (1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valentinamelica/R/Best-Practices-Parallelism/excel files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B450707D-2EA3-6C45-8F89-CC84D97BA57C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF75C08-65B7-2B45-807B-4192DBFAD1BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="860" yWindow="500" windowWidth="27940" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Data entry_merged'!$A$1:$AC$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Data entry_merged_filtered'!$A$1:$AE$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Data entry_merged_filtered'!$A$1:$AF$141</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -125,7 +125,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4775" uniqueCount="1198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4797" uniqueCount="1202">
   <si>
     <t>Reference number in Dr. Palme list</t>
   </si>
@@ -3850,6 +3850,18 @@
   </si>
   <si>
     <t>Decriptive stas-CV</t>
+  </si>
+  <si>
+    <t>Slopes comparison</t>
+  </si>
+  <si>
+    <t>Descriptive</t>
+  </si>
+  <si>
+    <t>Regression analysis</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -32832,7 +32844,9 @@
     <col min="22" max="22" width="23.1640625" style="16" customWidth="1"/>
     <col min="23" max="23" width="13.6640625" style="16" customWidth="1"/>
     <col min="24" max="24" width="9.83203125" style="16" customWidth="1"/>
-    <col min="25" max="32" width="27.83203125" style="16" customWidth="1"/>
+    <col min="25" max="25" width="27.83203125" style="16" customWidth="1"/>
+    <col min="26" max="31" width="27.83203125" style="16" hidden="1" customWidth="1"/>
+    <col min="32" max="32" width="27.83203125" style="16" customWidth="1"/>
     <col min="33" max="33" width="27.83203125" style="5"/>
     <col min="34" max="16384" width="27.83203125" style="16"/>
   </cols>
@@ -33226,7 +33240,9 @@
         <v>43</v>
       </c>
       <c r="AE5" s="14"/>
-      <c r="AF5" s="93"/>
+      <c r="AF5" t="s">
+        <v>1198</v>
+      </c>
     </row>
     <row r="6" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
@@ -33970,7 +33986,9 @@
       <c r="AC15" s="21"/>
       <c r="AD15" s="21"/>
       <c r="AE15" s="21"/>
-      <c r="AF15" s="93"/>
+      <c r="AF15" t="s">
+        <v>1198</v>
+      </c>
     </row>
     <row r="16" spans="1:33" s="54" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
@@ -34056,7 +34074,9 @@
       <c r="AC16" s="14"/>
       <c r="AD16" s="14"/>
       <c r="AE16" s="14"/>
-      <c r="AF16" s="93"/>
+      <c r="AF16" t="s">
+        <v>1198</v>
+      </c>
       <c r="AG16" s="5"/>
     </row>
     <row r="17" spans="1:33" s="54" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -34428,7 +34448,9 @@
       <c r="AC21" s="14"/>
       <c r="AD21" s="14"/>
       <c r="AE21" s="14"/>
-      <c r="AF21" s="93"/>
+      <c r="AF21" s="93" t="s">
+        <v>1201</v>
+      </c>
     </row>
     <row r="22" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
@@ -34727,7 +34749,9 @@
       <c r="AC25" s="14"/>
       <c r="AD25" s="14"/>
       <c r="AE25" s="14"/>
-      <c r="AF25" s="93"/>
+      <c r="AF25" s="93" t="s">
+        <v>1201</v>
+      </c>
     </row>
     <row r="26" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
@@ -35167,7 +35191,9 @@
       <c r="AC31" s="14"/>
       <c r="AD31" s="14"/>
       <c r="AE31" s="14"/>
-      <c r="AF31" s="93"/>
+      <c r="AF31" t="s">
+        <v>1198</v>
+      </c>
       <c r="AG31" s="5"/>
     </row>
     <row r="32" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -35324,7 +35350,9 @@
       <c r="AC33" s="26"/>
       <c r="AD33" s="26"/>
       <c r="AE33" s="26"/>
-      <c r="AF33" s="93"/>
+      <c r="AF33" s="93" t="s">
+        <v>1201</v>
+      </c>
     </row>
     <row r="34" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
@@ -35552,7 +35580,9 @@
       <c r="AC36" s="14"/>
       <c r="AD36" s="14"/>
       <c r="AE36" s="14"/>
-      <c r="AF36" s="93"/>
+      <c r="AF36" t="s">
+        <v>1198</v>
+      </c>
       <c r="AG36" s="5"/>
     </row>
     <row r="37" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -36011,7 +36041,9 @@
       <c r="AC42" s="14"/>
       <c r="AD42" s="14"/>
       <c r="AE42" s="14"/>
-      <c r="AF42" s="93"/>
+      <c r="AF42" s="93" t="s">
+        <v>1201</v>
+      </c>
     </row>
     <row r="43" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
@@ -36167,7 +36199,9 @@
       <c r="AC44" s="14"/>
       <c r="AD44" s="14"/>
       <c r="AE44" s="14"/>
-      <c r="AF44" s="93"/>
+      <c r="AF44" t="s">
+        <v>1200</v>
+      </c>
     </row>
     <row r="45" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
@@ -36251,7 +36285,9 @@
       <c r="AC45" s="14"/>
       <c r="AD45" s="14"/>
       <c r="AE45" s="14"/>
-      <c r="AF45" s="93"/>
+      <c r="AF45" t="s">
+        <v>1198</v>
+      </c>
     </row>
     <row r="46" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
@@ -36553,7 +36589,9 @@
       </c>
       <c r="AD49" s="14"/>
       <c r="AE49" s="14"/>
-      <c r="AF49" s="93"/>
+      <c r="AF49" t="s">
+        <v>1198</v>
+      </c>
     </row>
     <row r="50" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
@@ -37360,7 +37398,9 @@
       <c r="AC60" s="14"/>
       <c r="AD60" s="14"/>
       <c r="AE60" s="14"/>
-      <c r="AF60" s="93"/>
+      <c r="AF60" t="s">
+        <v>1198</v>
+      </c>
     </row>
     <row r="61" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
@@ -37588,7 +37628,9 @@
       <c r="AC63" s="14"/>
       <c r="AD63" s="14"/>
       <c r="AE63" s="14"/>
-      <c r="AF63" s="93"/>
+      <c r="AF63" s="93" t="s">
+        <v>1201</v>
+      </c>
     </row>
     <row r="64" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2">
@@ -37816,7 +37858,9 @@
       <c r="AC66" s="14"/>
       <c r="AD66" s="14"/>
       <c r="AE66" s="14"/>
-      <c r="AF66" s="93"/>
+      <c r="AF66" t="s">
+        <v>1198</v>
+      </c>
     </row>
     <row r="67" spans="1:33" s="34" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2">
@@ -38415,7 +38459,9 @@
       <c r="AC74" s="14"/>
       <c r="AD74" s="14"/>
       <c r="AE74" s="14"/>
-      <c r="AF74" s="93"/>
+      <c r="AF74" t="s">
+        <v>1198</v>
+      </c>
     </row>
     <row r="75" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="2">
@@ -38649,7 +38695,9 @@
       <c r="AC77" s="14"/>
       <c r="AD77" s="14"/>
       <c r="AE77" s="14"/>
-      <c r="AF77" s="93"/>
+      <c r="AF77" t="s">
+        <v>1198</v>
+      </c>
     </row>
     <row r="78" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="2">
@@ -38875,7 +38923,9 @@
       <c r="AC80" s="14"/>
       <c r="AD80" s="14"/>
       <c r="AE80" s="14"/>
-      <c r="AF80" s="93"/>
+      <c r="AF80" t="s">
+        <v>1200</v>
+      </c>
     </row>
     <row r="81" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="2">
@@ -39969,7 +40019,9 @@
       </c>
       <c r="AD95" s="14"/>
       <c r="AE95" s="14"/>
-      <c r="AF95" s="93"/>
+      <c r="AF95" t="s">
+        <v>1198</v>
+      </c>
     </row>
     <row r="96" spans="1:32" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="2">
@@ -40195,7 +40247,9 @@
       <c r="AC98" s="14"/>
       <c r="AD98" s="14"/>
       <c r="AE98" s="14"/>
-      <c r="AF98" s="93"/>
+      <c r="AF98" s="93" t="s">
+        <v>1201</v>
+      </c>
     </row>
     <row r="99" spans="1:32" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="2">
@@ -42083,7 +42137,9 @@
       <c r="AC124" s="14"/>
       <c r="AD124" s="14"/>
       <c r="AE124" s="14"/>
-      <c r="AF124" s="93"/>
+      <c r="AF124" t="s">
+        <v>1198</v>
+      </c>
     </row>
     <row r="125" spans="1:33" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="2">
@@ -42317,7 +42373,9 @@
       <c r="AC127" s="14"/>
       <c r="AD127" s="14"/>
       <c r="AE127" s="14"/>
-      <c r="AF127" s="93"/>
+      <c r="AF127" s="93" t="s">
+        <v>1199</v>
+      </c>
     </row>
     <row r="128" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="2">
@@ -65510,7 +65568,7 @@
       <c r="AF994" s="14"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AE141" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AF141" xr:uid="{58C4E5A1-DE9F-40CA-8EF9-C58D61B2370B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AG994">
     <sortCondition ref="L2:L994"/>
     <sortCondition ref="M2:M994"/>

</xml_diff>